<commit_message>
feat(referencias): substitui citacoes genericas por capitulo verificado em 801 questoes
Antes: descritor de assunto nas autorais e 'Miller 9th; Barash; Morgan' repetido
em 62 das 80 questoes do TEA 2023, sem capitulo nem pagina — citacao inverificavel.

- Sumarios extraidos dos marcadores de 5 obras e conferidos contra as paginas de
  abertura: SAESP 10ed (230 caps), Miller 10ed (87), Guyton 14ed (85),
  Stoelting's 6ed (47) e Peripheral Nerve Blocks US-guided (40)
- Cada capitulo citado foi confirmado por busca de termos no texto do PDF,
  nao escolhido pelo titulo nem citado de memoria
- 796 questoes citam o SAESP; 215 ganham segunda obra onde ela aprofunda
- Sem numero de pagina: os PDFs nao tem numeracao impressa recuperavel,
  entao a unidade citavel confiavel e o capitulo
- 2 questoes ficam sem referencia por lacuna real das obras
- Espelhado nas planilhas de origem, senao reimportar desfaria tudo

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/TEA_2023_importacao_comentada_com_niveis_ia.xlsx
+++ b/exports/TEA_2023_importacao_comentada_com_niveis_ia.xlsx
@@ -621,7 +621,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Código Civil Brasileiro, art. 951; Código de Ética Médica, CFM.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 3: Legislação Aplicada à Prática da Anestesiologia</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Sociedade Brasileira de Anestesiologia. Estatuto Social e documentos institucionais.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 2: As Associações de Anestesiologistas no Brasil e no Mundo</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash Clinical Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 5: Risco Profissional do Anestesiologista e Transtorno de Uso de Susbstâncias</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 72: Avaliação e Condutas Pré-anestésicas</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 72: Avaliação e Condutas Pré-anestésicas</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 68: Via Aérea Difícil</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 23: Anatomia do Sistema Respiratório</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 86: Monitorização do Sistema Nervoso • Miller's Anesthesia, 10ª ed. — cap. 30: Patient Positioning and Associated Risks</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 171: Anestesia para Cirurgias da Coluna</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 85: Princípios da Monitorização e Instrumentação Intraoperatória</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 87: Monitorização do Sistema Respiratório</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 87: Monitorização do Sistema Respiratório</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 21: Anatomia e Fisiologia do Sistema Nervoso Autônomo • Guyton &amp; Hall, Tratado de Fisiologia Médica, 14ª ed. — cap. 61: Sistema Nervoso Autônomo e Medula Adrenal</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 172: Fatores Determinantes das Pressões Intracranianas e de Perfusão Encefálica • Miller's Anesthesia, 10ª ed. — cap. 10: Cerebral Physiology and the Effects of Anesthetic Drugs</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 49: Antagonistas Adrenérgicos</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 51: Arritmias Cardíacas e Tratamento Farmacológico</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 24: Mecânica Respiratória e Controle da Respiração • Guyton &amp; Hall, Tratado de Fisiologia Médica, 14ª ed. — cap. 38: Ventilação Pulmonar</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 23: Anatomia do Sistema Respiratório • Guyton &amp; Hall, Tratado de Fisiologia Médica, 14ª ed. — cap. 38: Ventilação Pulmonar</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 38: Conceitos Farmacocinéticos e Farmacodinâmicos • Stoelting's Pharmacology &amp; Physiology in Anesthetic Practice, 6ª ed. — cap. 2: Basic Principles of Pharmacology</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 101: Anestesia Venosa Total Luiz Eduardo de Paula Gomes Miziara • Miller's Anesthesia, 10ª ed. — cap. 23: Intravenous Drug Delivery Systems</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 44: Hipnóticos: Propofol, Etomidato, Cetamina e Alfa 2 Agonistas • Miller's Anesthesia, 10ª ed. — cap. 21: Intravenous Anesthetics</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 44: Hipnóticos: Propofol, Etomidato, Cetamina e Alfa 2 Agonistas • Miller's Anesthesia, 10ª ed. — cap. 21: Intravenous Anesthetics</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 41: Farmacocinética dos Anestésicos Inalatórios • Miller's Anesthesia, 10ª ed. — cap. 18: Inhaled Anesthetic Uptake, Distribution, Metabolism, and Toxicity</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 41: Farmacocinética dos Anestésicos Inalatórios • Miller's Anesthesia, 10ª ed. — cap. 18: Inhaled Anesthetic Uptake, Distribution, Metabolism, and Toxicity</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 42: Anestésicos Locais • Peripheral Nerve Blocks and Anatomy for Ultrasound-Guided Regional Anesthesia (2021) — cap. 2: Local Anesthetics: Clinical Pharmacology and Selection</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 42: Anestésicos Locais • Peripheral Nerve Blocks and Anatomy for Ultrasound-Guided Regional Anesthesia (2021) — cap. 2: Local Anesthetics: Clinical Pharmacology and Selection</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 53: Bloqueadores Neuromusculares e Antagonistas • Stoelting's Pharmacology &amp; Physiology in Anesthetic Practice, 6ª ed. — cap. 12: Neuromuscular-Blocking Drugs and Reversal Agents</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 22: Fisiologia da Função Neuromuscular • Miller's Anesthesia, 10ª ed. — cap. 31: Neuromuscular Disorders and Other Genetic Disorders</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>American Heart Association. Guidelines for CPR and ECC; Morgan &amp; Mikhail, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 201: Reanimação Cardiorrespiratória no Adulto</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>American Heart Association. Guidelines for CPR and ECC; Morgan &amp; Mikhail, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 201: Reanimação Cardiorrespiratória no Adulto</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 106: Anestesia Peridural Bruno Erick Sinedino de Araújo • Miller's Anesthesia, 10ª ed. — cap. 41: Spinal, Epidural, and Caudal Anesthesia</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 103: Elementos de Anatomia: Ressonância Nuclear Magnética e Tomografia Computadorizada • Miller's Anesthesia, 10ª ed. — cap. 52: Anesthesia for Vascular Surgery</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 53: Bloqueadores Neuromusculares e Antagonistas • Miller's Anesthesia, 10ª ed. — cap. 39: Neuromuscular Monitoring</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 125: Eventos Adversos na Recuperação Pós-Anestésica</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash Clinical Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 227: Tipos de Estudo e Planejamento de Pesquisa</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 87: Monitorização do Sistema Respiratório</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 61: Vaporizadores e Fluxômetros</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 60: Componenetes dos Aparelhos de Anestesia</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 40: Anestésicos Inalatórios • Miller's Anesthesia, 10ª ed. — cap. 17: Inhaled Anesthetics: Mechanisms of Action</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 190: Anestesia para Eletroconvulsoterapia Julio Cesar Mercador de Freitas</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 113: Anestesia Regional Intravenosa Leonardo de Andrade Reis • Miller's Anesthesia, 10ª ed. — cap. 25: Local Anesthetics</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 104: Bloqueios Regionais Guiados pela Ultrassonografia • Peripheral Nerve Blocks and Anatomy for Ultrasound-Guided Regional Anesthesia (2021) — cap. 6: Monitoring and Documentation in Regional Anesthesia</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 95: Equilíbrio Ácido-base e Hidroeletrolítico</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 98: Terapia de Fluidos Perioperatória</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; diretrizes de reversão de anticoagulantes.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 57: Anticoagulantes e Antiagregantes Plaquetários</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 76: Avaliação do Sistema Renal • Miller's Anesthesia, 10ª ed. — cap. 55: Anesthesia and the Renal and Genitourinary Systems</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.; referências de anestesia urológica.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 167: Anestesia para Litotripsia Extracorpórea por Ondas de Choque</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Chestnut's Obstetric Anesthesia, 6th ed.; Miller's Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 128: Analgesia Para o Trabalho de Parto</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Chestnut's Obstetric Anesthesia, 6th ed.; Miller's Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 128: Analgesia Para o Trabalho de Parto</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 171: Anestesia para Cirurgias da Coluna</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 163: Anestesia para Cirurgia Videolaparoscópica e Robótica</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 183: Anestesia para Cirurgias Orais, Nasais, Seios da Face e Ouvidos</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 181: Anestesia em Oftalmologia: Fisiologia Ocular e</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 185: Anestesia Ambulatorial</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 124: Estágios da Recuperação da Anestesia: Aspectos Clínicos e Critérios de Alta André de Moraes Porto</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 37: Resposta Neuroendócrina, Imunológica e Metabólica ao Trauma Cirúrgico • Miller's Anesthesia, 10ª ed. — cap. 41: Spinal, Epidural, and Caudal Anesthesia</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 72: Avaliação e Condutas Pré-anestésicas</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 82: Jejum Pré-anestésico e Avaliação do Conteúdo Gástrico</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -5319,7 +5319,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 209: Fisiopatologia do Estado de Choque</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -5400,7 +5400,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 176: Anestesia no Trauma Cranioencefálico</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 91: Monitorização do Sistema Endócrino</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 169: Anestesia para Cirurgias Ortopédicas dos Membros Superiores • Peripheral Nerve Blocks and Anatomy for Ultrasound-Guided Regional Anesthesia (2021) — cap. 8: Continuous Peripheral Nerve Blocks</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 178: Anestesia para Cirurgia Bucomaxilofacial</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -5724,7 +5724,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 149: Ventilação Monopulmonar</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 155: Anestesia para Cirurgia Valvar</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 153: Circulação Extracorpórea e Assistência Circulatória Mecânica</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 173: Anestesia para Cirurgia de Tumores Cerebrais Christiano dos Santos e Santos</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -6048,7 +6048,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 94: Regulação e Monitorização da Temperatura</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; textos de medicina perioperatória e choque.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 215: Avaliação e Abordagem do Paciente Politraumatizado</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; textos de medicina perioperatória e choque.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 209: Fisiopatologia do Estado de Choque</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 82: Jejum Pré-anestésico e Avaliação do Conteúdo Gástrico</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>A Practice of Anesthesia for Infants and Children, 7th ed.; Morgan &amp; Mikhail, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 145: Reposição Volêmica e Hemotransfusão em</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>A Practice of Anesthesia for Infants and Children, 7th ed.; Morgan &amp; Mikhail, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 143: Anestesia Regional em Pediatria</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 186: Anestesia para Radiodiagnóstico Antônio Márcio de Sanfim Arantes Pereira</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
@@ -6615,7 +6615,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash Clinical Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 116: Avaliação e Tratamento da Dor Aguda</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash Clinical Anesthesia, 9th ed.</t>
+          <t>Miller's Anesthesia, 10ª ed. — cap. 28: Preoperative Evaluation</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
@@ -6777,7 +6777,7 @@
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 60: Componenetes dos Aparelhos de Anestesia</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash Clinical Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 10: Segurança do Paciente na Anestesia</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash Clinical Anesthesia, 9th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 6: Fundamentos de Organização e Gestão para Serviços de Anestesia</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>Miller's Anesthesia, 9th ed.; Barash, Cullen and Stoelting's Clinical Anesthesia, 9th ed.; Morgan &amp; Mikhail's Clinical Anesthesiology, 7th ed.</t>
+          <t>SAESP, Tratado de Anestesiologia, 10ª ed. — cap. 92: Monitorização do Sistema Hematológico</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">

</xml_diff>